<commit_message>
Calculators - OD680 non-linearity correction for FMT-150
</commit_message>
<xml_diff>
--- a/website/static/files/SigmaII_example.xlsx
+++ b/website/static/files/SigmaII_example.xlsx
@@ -5,19 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zavrel.t\Dropbox\Programming\Python\Flask_server\website\static\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zavre\Dropbox\Programming\Python\Flask_server\website\static\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D876E1-6759-44A2-A213-89997F6032E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC18618-2A52-46D4-8872-CB283CD50A55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{005EB3D4-D238-4DE0-AD51-3D8ECF08E4BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{005EB3D4-D238-4DE0-AD51-3D8ECF08E4BD}"/>
   </bookViews>
   <sheets>
-    <sheet name="SigmaII_04-200-01-2" sheetId="2" r:id="rId1"/>
-    <sheet name="List1" sheetId="1" r:id="rId2"/>
+    <sheet name="SigmaII" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'SigmaII_04-200-01-2'!$A$1:$M$7</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">SigmaII!$A$1:$M$7</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -311,11 +310,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -462,7 +460,7 @@
           </c:errBars>
           <c:xVal>
             <c:numRef>
-              <c:f>'SigmaII_04-200-01-2'!$J$13:$J$17</c:f>
+              <c:f>SigmaII!$J$13:$J$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -486,7 +484,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SigmaII_04-200-01-2'!$K$13:$K$17</c:f>
+              <c:f>SigmaII!$K$13:$K$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -2070,40 +2068,40 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" t="s">
         <v>17</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="M2" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2111,40 +2109,40 @@
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" t="s">
         <v>27</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" t="s">
         <v>28</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="M3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2152,40 +2150,40 @@
       <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" t="s">
         <v>24</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" t="s">
         <v>35</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" t="s">
         <v>36</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="L4" t="s">
         <v>37</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="M4" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2193,40 +2191,40 @@
       <c r="A5">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" t="s">
         <v>42</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" t="s">
         <v>43</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" t="s">
         <v>44</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" t="s">
         <v>45</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" t="s">
         <v>46</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" t="s">
         <v>47</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="L5" t="s">
         <v>48</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="M5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2234,40 +2232,40 @@
       <c r="A6">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" t="s">
         <v>56</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" t="s">
         <v>57</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" t="s">
         <v>58</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" t="s">
         <v>59</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="M6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2275,40 +2273,40 @@
       <c r="A7">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>62</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" t="s">
         <v>63</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" t="s">
         <v>64</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" t="s">
         <v>24</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" t="s">
         <v>65</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" t="s">
         <v>66</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" t="s">
         <v>67</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L7" t="s">
         <v>68</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="M7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2316,7 +2314,7 @@
       <c r="J13">
         <v>440</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>0.75900000000000001</v>
       </c>
     </row>
@@ -2324,7 +2322,7 @@
       <c r="J14">
         <v>480</v>
       </c>
-      <c r="K14" s="3">
+      <c r="K14" s="2">
         <v>0.24199999999999999</v>
       </c>
     </row>
@@ -2332,7 +2330,7 @@
       <c r="J15">
         <v>540</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>0.78100000000000003</v>
       </c>
     </row>
@@ -2340,7 +2338,7 @@
       <c r="J16">
         <v>590</v>
       </c>
-      <c r="K16" s="3">
+      <c r="K16" s="2">
         <v>3.782</v>
       </c>
     </row>
@@ -2348,7 +2346,7 @@
       <c r="J17">
         <v>625</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>7</v>
       </c>
     </row>
@@ -2358,15 +2356,6 @@
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DDBA9A9-892F-4724-88DC-7D3DC8556965}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>